<commit_message>
Add CR-aware reconciliation workbook and scope-management skill history
- New CR-aware xlsx overlay covering CR01, CR02, and Project Evolution
- Updated Finalised workbook with CR-aware revisions
- CR source extracts and build scripts for reproducibility
- History updated with 2026-04-17 skill-authoring session (ART-2057/2058/2059)
</commit_message>
<xml_diff>
--- a/docs/Hireup Scope Analysis — Finalised.xlsx
+++ b/docs/Hireup Scope Analysis — Finalised.xlsx
@@ -604,6 +604,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
@@ -639,11 +641,11 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>65%</t>
+          <t>66%</t>
         </is>
       </c>
     </row>
@@ -658,7 +660,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>19%</t>
         </is>
       </c>
     </row>
@@ -684,7 +686,7 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
@@ -692,6 +694,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -852,6 +855,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
@@ -968,6 +972,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
@@ -1098,6 +1103,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
@@ -1211,6 +1217,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
@@ -1331,6 +1338,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
@@ -1461,6 +1469,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
@@ -1569,7 +1578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5695,6 +5704,90 @@
       <c r="H98" s="9" t="inlineStr">
         <is>
           <t>RW backs dedicated codes; GL mapping is the extension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>PAYM-176</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>2c9 Prod Instance set up</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>In Scope</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>SOW 3.3 (Installation and Configuration)</t>
+        </is>
+      </c>
+      <c r="H99" s="7" t="inlineStr">
+        <is>
+          <t>Production org setup with 2cloudnine packages + Hireup custom flows. Core deployment activity — Guy confirmed packages installed 9 Feb; Heidi marked Done 16 Apr (core config complete). Added via verification against Jira report 20260414 PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>PAYM-277</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>Broken Shift Allowance not triggered when first shift crosses midnight</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>Not a bug</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>In Scope</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>SOW Gap 3 (Broken Shift); 18 Feb 2026 workshop decision</t>
+        </is>
+      </c>
+      <c r="H100" s="7" t="inlineStr">
+        <is>
+          <t>Resolved 'Not a bug' 2 Apr 2026. Hireup attempted to re-litigate calendar-day broken-shift logic as rolling-12-hour. Heidi's 1 Apr comment: 'agreed by all on 18 Feb to use calendar day — highly significant change in scope. If rolling 12-hour is now needed, raise as formal CR.' Scope line held — no commercial impact. Added via verification against Jira report 20260414 PDF.</t>
         </is>
       </c>
     </row>
@@ -7196,6 +7289,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -7226,7 +7320,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>97 JIRA tickets classified against SOW (Aug 2025), Requirements Workbook, Discovery Workbook, RAID Log, and Project Timeline.</t>
+          <t>99 JIRA tickets classified against SOW (Aug 2025), Requirements Workbook, Discovery Workbook, RAID Log, and Project Timeline. (Initial pass: 97 tickets from JIRA.xml; 2 additional tickets — PAYM-176, PAYM-277 — added 17 Apr after PDF cross-check.)</t>
         </is>
       </c>
     </row>
@@ -7266,6 +7360,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -7364,6 +7459,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
@@ -7496,6 +7592,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
@@ -7590,6 +7687,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
@@ -7682,7 +7780,7 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>JIRA.xml (97 tickets from PAYM project)</t>
+          <t>JIRA.xml (138 keys, 97 in-scope PAYM tickets) + JIRA (2).xml verification export (17 Apr 2026) — added PAYM-176 and PAYM-277 after cross-check against Jira report 20260414 PDF.</t>
         </is>
       </c>
     </row>

</xml_diff>